<commit_message>
Change: Spring zu Springboot
</commit_message>
<xml_diff>
--- a/Technologieauswahk.xlsx
+++ b/Technologieauswahk.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28803"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
   <workbookPr showInkAnnotation="0"/>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{ABC4BEC5-E699-374D-ACBA-EC645EBA4F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61BBEA9F-B488-49F8-A2CC-719AC7C33CCE}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/justpna/Library/Mobile Documents/com~apple~CloudDocs/Cloud/FH Dortmund/S4/SWT2/sonar/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9CA96E9-152A-204F-99DE-64397AFB60BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -57,9 +62,6 @@
     <t>Entwicklungswerkzeuge Backend</t>
   </si>
   <si>
-    <t>Spring</t>
-  </si>
-  <si>
     <t>NodeJS</t>
   </si>
   <si>
@@ -166,6 +168,9 @@
   </si>
   <si>
     <t>5. Sicherheit</t>
+  </si>
+  <si>
+    <t>Springboot</t>
   </si>
 </sst>
 </file>
@@ -175,7 +180,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -784,19 +789,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{770A1D49-1822-B34A-AE6E-85391E6FD248}">
   <dimension ref="A1:AG44"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -804,7 +809,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>1</v>
       </c>
@@ -812,7 +817,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2</v>
       </c>
@@ -820,7 +825,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>3</v>
       </c>
@@ -828,7 +833,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>4</v>
       </c>
@@ -836,61 +841,61 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.75" thickBot="1">
+    <row r="9" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="E10" s="10" t="s">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" t="s">
+        <v>8</v>
+      </c>
+      <c r="I10" t="s">
         <v>9</v>
       </c>
-      <c r="I10" t="s">
+      <c r="K10" t="s">
         <v>10</v>
       </c>
-      <c r="K10" t="s">
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C11" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>12</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="F11" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="G11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" t="s">
         <v>15</v>
       </c>
-      <c r="G11" t="s">
+      <c r="I11" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" t="s">
         <v>14</v>
       </c>
-      <c r="H11" t="s">
+      <c r="K11" t="s">
+        <v>13</v>
+      </c>
+      <c r="L11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+      <c r="C12" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="I11" t="s">
-        <v>14</v>
-      </c>
-      <c r="J11" t="s">
-        <v>15</v>
-      </c>
-      <c r="K11" t="s">
-        <v>14</v>
-      </c>
-      <c r="L11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="C12" s="3" t="s">
-        <v>17</v>
       </c>
       <c r="D12" s="3">
         <v>7.6E-3</v>
@@ -924,9 +929,9 @@
         <v>7.6E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:12">
+    <row r="13" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="C13" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D13" s="2">
         <v>6.8199999999999997E-2</v>
@@ -960,9 +965,9 @@
         <v>0.13639999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:12">
+    <row r="14" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="C14" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D14" s="3">
         <v>7.5800000000000006E-2</v>
@@ -996,9 +1001,9 @@
         <v>0.30320000000000003</v>
       </c>
     </row>
-    <row r="15" spans="1:12">
+    <row r="15" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="C15" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D15" s="3">
         <v>0.1061</v>
@@ -1032,9 +1037,9 @@
         <v>0.31830000000000003</v>
       </c>
     </row>
-    <row r="16" spans="1:12">
+    <row r="16" spans="1:12" ht="16" x14ac:dyDescent="0.2">
       <c r="C16" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D16" s="2">
         <v>0.1515</v>
@@ -1068,9 +1073,9 @@
         <v>0.60599999999999998</v>
       </c>
     </row>
-    <row r="17" spans="3:33">
+    <row r="17" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C17" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17" s="3">
         <v>0.1515</v>
@@ -1104,9 +1109,9 @@
         <v>0.60599999999999998</v>
       </c>
     </row>
-    <row r="18" spans="3:33">
+    <row r="18" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C18" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D18" s="2">
         <v>5.2999999999999999E-2</v>
@@ -1140,9 +1145,9 @@
         <v>0.21199999999999999</v>
       </c>
     </row>
-    <row r="19" spans="3:33" ht="15.75" thickBot="1">
+    <row r="19" spans="3:33" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C19" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D19" s="3">
         <v>9.8500000000000004E-2</v>
@@ -1176,9 +1181,9 @@
         <v>0.29549999999999998</v>
       </c>
     </row>
-    <row r="20" spans="3:33" ht="15.75" thickBot="1">
+    <row r="20" spans="3:33" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C20" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D20" s="5">
         <f>SUM(D12:D19)</f>
@@ -1202,9 +1207,9 @@
         <v>2.4850000000000003</v>
       </c>
     </row>
-    <row r="22" spans="3:33">
+    <row r="22" spans="3:33" x14ac:dyDescent="0.2">
       <c r="R22" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="S22" s="13"/>
       <c r="T22" s="14">
@@ -1249,16 +1254,16 @@
         <v>#REF!</v>
       </c>
       <c r="AG22" s="16" t="e">
-        <f>AF22</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="23" spans="3:33">
+        <f t="shared" ref="AG22:AG33" si="4">AF22</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="23" spans="3:33" x14ac:dyDescent="0.2">
       <c r="E23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="R23" s="17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S23" s="18">
         <v>0</v>
@@ -1303,26 +1308,26 @@
         <v>#REF!</v>
       </c>
       <c r="AG23" s="20" t="e">
-        <f>AF23</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="24" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="24" spans="3:33" x14ac:dyDescent="0.2">
       <c r="E24" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" t="s">
+        <v>28</v>
+      </c>
+      <c r="I24" t="s">
         <v>29</v>
       </c>
-      <c r="I24" t="s">
+      <c r="K24" t="s">
         <v>30</v>
       </c>
-      <c r="K24" t="s">
-        <v>31</v>
-      </c>
       <c r="R24" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S24" s="14">
         <v>0</v>
@@ -1367,43 +1372,43 @@
         <v>#REF!</v>
       </c>
       <c r="AG24" s="16" t="e">
-        <f>AF24</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="25" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="25" spans="3:33" x14ac:dyDescent="0.2">
       <c r="C25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" t="s">
         <v>12</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E25" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="F25" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="G25" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" t="s">
         <v>15</v>
       </c>
-      <c r="G25" t="s">
+      <c r="I25" t="s">
+        <v>13</v>
+      </c>
+      <c r="J25" t="s">
         <v>14</v>
       </c>
-      <c r="H25" t="s">
-        <v>16</v>
-      </c>
-      <c r="I25" t="s">
+      <c r="K25" t="s">
+        <v>13</v>
+      </c>
+      <c r="L25" t="s">
         <v>14</v>
       </c>
-      <c r="J25" t="s">
-        <v>15</v>
-      </c>
-      <c r="K25" t="s">
-        <v>14</v>
-      </c>
-      <c r="L25" t="s">
-        <v>15</v>
-      </c>
       <c r="R25" s="17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="S25" s="18">
         <v>0</v>
@@ -1448,13 +1453,13 @@
         <v>#REF!</v>
       </c>
       <c r="AG25" s="20" t="e">
-        <f>AF25</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="26" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="26" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C26" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D26" s="2">
         <v>0.1515</v>
@@ -1488,7 +1493,7 @@
         <v>0.60599999999999998</v>
       </c>
       <c r="R26" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="S26" s="14">
         <v>0</v>
@@ -1533,13 +1538,13 @@
         <v>#REF!</v>
       </c>
       <c r="AG26" s="16" t="e">
-        <f>AF26</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="27" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="27" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C27" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D27" s="3">
         <v>7.6E-3</v>
@@ -1548,32 +1553,32 @@
         <v>3</v>
       </c>
       <c r="F27" s="8">
-        <f t="shared" ref="F27:F31" si="4">D27*E27</f>
+        <f t="shared" ref="F27:F31" si="5">D27*E27</f>
         <v>2.2800000000000001E-2</v>
       </c>
       <c r="G27">
         <v>2</v>
       </c>
       <c r="H27">
-        <f t="shared" ref="H27:H31" si="5">D27*G27</f>
+        <f t="shared" ref="H27:H31" si="6">D27*G27</f>
         <v>1.52E-2</v>
       </c>
       <c r="I27">
         <v>1</v>
       </c>
       <c r="J27">
-        <f t="shared" ref="J27:J31" si="6">D27*I27</f>
+        <f t="shared" ref="J27:J31" si="7">D27*I27</f>
         <v>7.6E-3</v>
       </c>
       <c r="K27">
         <v>2</v>
       </c>
       <c r="L27">
-        <f t="shared" ref="L27:L31" si="7">D27*K27</f>
+        <f t="shared" ref="L27:L31" si="8">D27*K27</f>
         <v>1.52E-2</v>
       </c>
       <c r="R27" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="S27" s="18">
         <v>0</v>
@@ -1618,13 +1623,13 @@
         <v>#REF!</v>
       </c>
       <c r="AG27" s="20" t="e">
-        <f>AF27</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="28" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="28" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C28" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D28" s="2">
         <v>6.8199999999999997E-2</v>
@@ -1633,32 +1638,32 @@
         <v>3</v>
       </c>
       <c r="F28" s="8">
-        <f t="shared" si="4"/>
-        <v>0.2046</v>
-      </c>
-      <c r="G28">
-        <v>3</v>
-      </c>
-      <c r="H28">
         <f t="shared" si="5"/>
         <v>0.2046</v>
       </c>
-      <c r="I28">
-        <v>3</v>
-      </c>
-      <c r="J28">
+      <c r="G28">
+        <v>3</v>
+      </c>
+      <c r="H28">
         <f t="shared" si="6"/>
         <v>0.2046</v>
       </c>
+      <c r="I28">
+        <v>3</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="7"/>
+        <v>0.2046</v>
+      </c>
       <c r="K28">
         <v>2</v>
       </c>
       <c r="L28">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.13639999999999999</v>
       </c>
       <c r="R28" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="S28" s="14">
         <v>1</v>
@@ -1703,13 +1708,13 @@
         <v>#REF!</v>
       </c>
       <c r="AG28" s="16" t="e">
-        <f>AF28</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="29" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="29" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C29" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D29" s="3">
         <v>7.5800000000000006E-2</v>
@@ -1718,32 +1723,32 @@
         <v>4</v>
       </c>
       <c r="F29" s="8">
-        <f t="shared" si="4"/>
-        <v>0.30320000000000003</v>
-      </c>
-      <c r="G29">
-        <v>4</v>
-      </c>
-      <c r="H29">
         <f t="shared" si="5"/>
         <v>0.30320000000000003</v>
       </c>
-      <c r="I29">
-        <v>4</v>
-      </c>
-      <c r="J29">
+      <c r="G29">
+        <v>4</v>
+      </c>
+      <c r="H29">
         <f t="shared" si="6"/>
         <v>0.30320000000000003</v>
       </c>
+      <c r="I29">
+        <v>4</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="7"/>
+        <v>0.30320000000000003</v>
+      </c>
       <c r="K29">
         <v>3</v>
       </c>
       <c r="L29">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.22740000000000002</v>
       </c>
       <c r="R29" s="17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="S29" s="18">
         <v>1</v>
@@ -1788,13 +1793,13 @@
         <v>#REF!</v>
       </c>
       <c r="AG29" s="20" t="e">
-        <f>AF29</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="30" spans="3:33" ht="29.25">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="30" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C30" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D30" s="2">
         <v>6.8199999999999997E-2</v>
@@ -1803,32 +1808,32 @@
         <v>4</v>
       </c>
       <c r="F30" s="8">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.27279999999999999</v>
       </c>
       <c r="G30">
         <v>3</v>
       </c>
       <c r="H30">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.2046</v>
       </c>
       <c r="I30">
         <v>4</v>
       </c>
       <c r="J30">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.27279999999999999</v>
       </c>
       <c r="K30">
         <v>2</v>
       </c>
       <c r="L30">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.13639999999999999</v>
       </c>
       <c r="R30" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="S30" s="14">
         <v>0</v>
@@ -1873,13 +1878,13 @@
         <v>#REF!</v>
       </c>
       <c r="AG30" s="16" t="e">
-        <f>AF30</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="31" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="31" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C31" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D31" s="3">
         <v>0.1061</v>
@@ -1888,32 +1893,32 @@
         <v>3</v>
       </c>
       <c r="F31" s="8">
-        <f t="shared" si="4"/>
-        <v>0.31830000000000003</v>
-      </c>
-      <c r="G31">
-        <v>3</v>
-      </c>
-      <c r="H31">
         <f t="shared" si="5"/>
         <v>0.31830000000000003</v>
       </c>
+      <c r="G31">
+        <v>3</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="6"/>
+        <v>0.31830000000000003</v>
+      </c>
       <c r="I31">
         <v>2</v>
       </c>
       <c r="J31">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.2122</v>
       </c>
       <c r="K31">
         <v>3</v>
       </c>
       <c r="L31">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.31830000000000003</v>
       </c>
       <c r="R31" s="17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="S31" s="18">
         <v>0</v>
@@ -1958,13 +1963,13 @@
         <v>#REF!</v>
       </c>
       <c r="AG31" s="20" t="e">
-        <f>AF31</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="32" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="32" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C32" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D32" s="5">
         <f>SUM(D26:D31)</f>
@@ -1988,7 +1993,7 @@
         <v>1.4397</v>
       </c>
       <c r="R32" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="S32" s="14">
         <v>0</v>
@@ -2033,13 +2038,13 @@
         <v>#REF!</v>
       </c>
       <c r="AG32" s="16" t="e">
-        <f>AF32</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="33" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="33" spans="3:33" x14ac:dyDescent="0.2">
       <c r="R33" s="17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S33" s="18">
         <v>0</v>
@@ -2084,13 +2089,13 @@
         <v>#REF!</v>
       </c>
       <c r="AG33" s="20" t="e">
-        <f>AF33</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="34" spans="3:33">
+        <f t="shared" si="4"/>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="34" spans="3:33" x14ac:dyDescent="0.2">
       <c r="R34" s="21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="S34" s="14"/>
       <c r="T34" s="14"/>
@@ -2117,61 +2122,61 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="36" spans="3:33">
+    <row r="36" spans="3:33" x14ac:dyDescent="0.2">
       <c r="E36" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="3:33" x14ac:dyDescent="0.2">
+      <c r="E37" s="10" t="s">
         <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="3:33">
-      <c r="E37" s="10" t="s">
-        <v>36</v>
       </c>
       <c r="F37" s="6"/>
       <c r="G37" t="s">
+        <v>36</v>
+      </c>
+      <c r="I37" t="s">
         <v>37</v>
       </c>
-      <c r="I37" t="s">
+      <c r="K37" t="s">
         <v>38</v>
       </c>
-      <c r="K37" t="s">
+    </row>
+    <row r="38" spans="3:33" x14ac:dyDescent="0.2">
+      <c r="C38" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" t="s">
+        <v>13</v>
+      </c>
+      <c r="H38" t="s">
+        <v>15</v>
+      </c>
+      <c r="I38" t="s">
+        <v>13</v>
+      </c>
+      <c r="J38" t="s">
+        <v>14</v>
+      </c>
+      <c r="K38" t="s">
+        <v>13</v>
+      </c>
+      <c r="L38" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="3:33" ht="16" x14ac:dyDescent="0.2">
+      <c r="C39" s="2" t="s">
         <v>39</v>
-      </c>
-    </row>
-    <row r="38" spans="3:33">
-      <c r="C38" t="s">
-        <v>12</v>
-      </c>
-      <c r="D38" t="s">
-        <v>13</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F38" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G38" t="s">
-        <v>14</v>
-      </c>
-      <c r="H38" t="s">
-        <v>16</v>
-      </c>
-      <c r="I38" t="s">
-        <v>14</v>
-      </c>
-      <c r="J38" t="s">
-        <v>15</v>
-      </c>
-      <c r="K38" t="s">
-        <v>14</v>
-      </c>
-      <c r="L38" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="39" spans="3:33">
-      <c r="C39" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="D39" s="2">
         <v>0.1515</v>
@@ -2205,9 +2210,9 @@
         <v>0.60599999999999998</v>
       </c>
     </row>
-    <row r="40" spans="3:33">
+    <row r="40" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C40" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D40" s="3">
         <v>3.7900000000000003E-2</v>
@@ -2216,34 +2221,34 @@
         <v>3</v>
       </c>
       <c r="F40" s="8">
-        <f t="shared" ref="F40:F43" si="8">D40*E40</f>
+        <f t="shared" ref="F40:F43" si="9">D40*E40</f>
         <v>0.11370000000000001</v>
       </c>
       <c r="G40">
         <v>2</v>
       </c>
       <c r="H40">
-        <f t="shared" ref="H40:H43" si="9">D40*G40</f>
+        <f t="shared" ref="H40:H43" si="10">D40*G40</f>
         <v>7.5800000000000006E-2</v>
       </c>
       <c r="I40">
         <v>1</v>
       </c>
       <c r="J40">
-        <f t="shared" ref="J40:J43" si="10">D40*I40</f>
+        <f t="shared" ref="J40:J43" si="11">D40*I40</f>
         <v>3.7900000000000003E-2</v>
       </c>
       <c r="K40">
         <v>2</v>
       </c>
       <c r="L40">
-        <f t="shared" ref="L40:L43" si="11">D40*K40</f>
+        <f t="shared" ref="L40:L43" si="12">D40*K40</f>
         <v>7.5800000000000006E-2</v>
       </c>
     </row>
-    <row r="41" spans="3:33">
+    <row r="41" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C41" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D41" s="2">
         <v>3.0300000000000001E-2</v>
@@ -2252,34 +2257,34 @@
         <v>3</v>
       </c>
       <c r="F41" s="8">
-        <f t="shared" si="8"/>
-        <v>9.0900000000000009E-2</v>
-      </c>
-      <c r="G41">
-        <v>3</v>
-      </c>
-      <c r="H41">
         <f t="shared" si="9"/>
         <v>9.0900000000000009E-2</v>
       </c>
-      <c r="I41">
-        <v>3</v>
-      </c>
-      <c r="J41">
+      <c r="G41">
+        <v>3</v>
+      </c>
+      <c r="H41">
         <f t="shared" si="10"/>
         <v>9.0900000000000009E-2</v>
       </c>
+      <c r="I41">
+        <v>3</v>
+      </c>
+      <c r="J41">
+        <f t="shared" si="11"/>
+        <v>9.0900000000000009E-2</v>
+      </c>
       <c r="K41">
         <v>2</v>
       </c>
       <c r="L41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>6.0600000000000001E-2</v>
       </c>
     </row>
-    <row r="42" spans="3:33">
+    <row r="42" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C42" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D42" s="3">
         <v>9.8500000000000004E-2</v>
@@ -2288,34 +2293,34 @@
         <v>4</v>
       </c>
       <c r="F42" s="8">
-        <f t="shared" si="8"/>
-        <v>0.39400000000000002</v>
-      </c>
-      <c r="G42">
-        <v>4</v>
-      </c>
-      <c r="H42">
         <f t="shared" si="9"/>
         <v>0.39400000000000002</v>
       </c>
-      <c r="I42">
-        <v>4</v>
-      </c>
-      <c r="J42">
+      <c r="G42">
+        <v>4</v>
+      </c>
+      <c r="H42">
         <f t="shared" si="10"/>
         <v>0.39400000000000002</v>
       </c>
+      <c r="I42">
+        <v>4</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="11"/>
+        <v>0.39400000000000002</v>
+      </c>
       <c r="K42">
         <v>3</v>
       </c>
       <c r="L42">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.29549999999999998</v>
       </c>
     </row>
-    <row r="43" spans="3:33">
+    <row r="43" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C43" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D43" s="2">
         <v>5.2999999999999999E-2</v>
@@ -2324,34 +2329,34 @@
         <v>4</v>
       </c>
       <c r="F43" s="8">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.21199999999999999</v>
       </c>
       <c r="G43">
         <v>3</v>
       </c>
       <c r="H43">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.159</v>
       </c>
       <c r="I43">
         <v>4</v>
       </c>
       <c r="J43">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.21199999999999999</v>
       </c>
       <c r="K43">
         <v>2</v>
       </c>
       <c r="L43">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.106</v>
       </c>
     </row>
-    <row r="44" spans="3:33">
+    <row r="44" spans="3:33" ht="16" x14ac:dyDescent="0.2">
       <c r="C44" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D44" s="5">
         <f>SUM(D39:D43)</f>

</xml_diff>